<commit_message>
fix(brainlift): stop parse_register ingesting the B-pass log header as a source row
</commit_message>
<xml_diff>
--- a/Alpha HS Writing Course 2026-27/BrainLift_Knowledge_Tree_Sources.xlsx
+++ b/Alpha HS Writing Course 2026-27/BrainLift_Knowledge_Tree_Sources.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1715,38 +1715,6 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Claim</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Authority</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Recovery type</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Category 7: Progression and Architecture</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1758,1808 +1726,1318 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Primary Source</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Grounds (claim / SPOV)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Reachable via</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Compiled into (artifacts)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Knowledge Tree Category</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Document Title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Filename</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Absolute Path</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Hyperlink (file://)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Size (KB)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Role in the BrainLift / Why cited</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>On disk?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1. Standards Backbone (ACC / union-of-states)</t>
+          <t>Texas Education Agency (TEA), TEKS English Language Arts and Reading Standards</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alpha Common Core — G9–12 Writing Standards Spine (v1)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>05_AlphaCommonCore_Writing_Spine.md</t>
+          <t>G9-G12 writing standards (STAAR English I/II alignment); TEKS-specific compositional progression</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\05_AlphaCommonCore_Writing_Spine.md</t>
+          <t>https://tea.texas.gov/about-tea/laws-and-rules/texas-administrative-code/19-tac-chapter-110</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>05_AlphaCommonCore_Writing_Spine.md</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>The ACC definition (&gt;=2-state union), the CCSS-superset claim, and the 'author once, tag many' mapper. Grounds SPOV Truth 1.</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, 02_deviation_states_deepdive.md</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Category 1: Standards Backbone</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Standards Backbone (ACC / union-of-states)</t>
+          <t>California Department of Education, Common Core State Standards for English Language Arts</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Phase 0 — G9-12 Writing Standards: CCSS Adherence Map</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01_ccss_adherence_map.md</t>
+          <t>CCSS-family hub standards (W.9-10.1-3, W.11-12.1-3); argument, explanatory, narrative modes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\01_ccss_adherence_map.md</t>
+          <t>https://www.cde.ca.gov/be/st/ss/documents/finalelaccssstandards.pdf</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>01_ccss_adherence_map.md</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>CCSS coverage baseline: 50 states + DC vs CCSS (15 verbatim / 22 derived / 14 deviation).</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, 05_AlphaCommonCore_Writing_Spine.md</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Category 1: Standards Backbone</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1. Standards Backbone (ACC / union-of-states)</t>
+          <t>New York State Education Department (NYSED), Next Generation English Language Arts Learning Standards</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Phase 0 — G9–12 Writing Standards Deep-Dive: Non-CCSS Deviation States</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>02_deviation_states_deepdive.md</t>
+          <t>NY-CCSS aligned standards (9-10W1-3, 11-12W1-3); source-based analytical writing emphasis</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\02_deviation_states_deepdive.md</t>
+          <t>https://www.nysed.gov/curriculum-instruction/new-york-state-next-generation-english-language-arts-learning-standards</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>02_deviation_states_deepdive.md</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Where core deviation states (TX/VA/FL/NE/OK/SC + GA/MN) diverge from the common core.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, 03_state_assessment_format_map.md</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Category 1: Standards Backbone</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1. Standards Backbone (ACC / union-of-states)</t>
+          <t>Florida Department of Education, B.E.S.T. Standards for ELA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Phase 0 — G9–12 Writing Sub-Skill Extraction: Alabama + Arkansas</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>06a_deviation_AL_AR.md</t>
+          <t>FL B.E.S.T. deviation from CCSS (argumentation-first G7-10, expository separate strand)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\06a_deviation_AL_AR.md</t>
+          <t>https://cpalmsmediaprod.blob.core.windows.net/uploads/docs/standards/best/la/elabeststandardsfinal2108.pdf</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>06a_deviation_AL_AR.md</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Deviation-state sub-skill extraction: AL, AR (part of the 14-state mapping).</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, 02_deviation_states_deepdive.md</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Category 1: Standards Backbone</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1. Standards Backbone (ACC / union-of-states)</t>
+          <t>Arkansas Department of Education, ELA Standards (2023)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Phase 0 — G9-12 Writing Standards: Non-CCSS Deviation States (Idaho &amp; Maine)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>06b_deviation_ID_ME.md</t>
+          <t>Arkansas CCSS-aligned standards (evidence-based argument G9-12)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\06b_deviation_ID_ME.md</t>
+          <t>https://dese.ade.arkansas.gov/Files/AR_2023_9-12_ELA_Standards_and_Notes_1.25_LS.pdf</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>06b_deviation_ID_ME.md</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Deviation-state sub-skill extraction: ID, ME.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, 06a_deviation_AL_AR.md</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Category 1: Standards Backbone</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1. Standards Backbone (ACC / union-of-states)</t>
+          <t>Virginia Department of Education, Standards of Learning (SOL) for English</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Phase 0 — G9-12 Writing Standards: Non-CCSS Deviation States (North Dakota &amp; Wisconsin)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>06c_deviation_ND_WI.md</t>
+          <t>Virginia deviation standards (two-tier claim hierarchy in persuasive writing)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\06c_deviation_ND_WI.md</t>
+          <t>https://www.doe.virginia.gov/teaching-learning-assessment/k-12-standards-instruction/english-reading-literacy/standards-of-learning/2024-english-standards-of-learning</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>06c_deviation_ND_WI.md</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Deviation-state sub-skill extraction: ND, WI.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, 02_deviation_states_deepdive.md</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Category 1: Standards Backbone</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1. Standards Backbone (ACC / union-of-states)</t>
+          <t>Texas Education Agency (TEA), STAAR English I/II Blueprint Schematic</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>G9-12 State Summative Writing Assessment: Format Map (50 States + DC + National Layer)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>03_state_assessment_format_map.md</t>
+          <t>G9/G10 ECR+SCR format; Organization &amp; Development (0-3) + Conventions (0-2) rubric; gating logic</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\03_state_assessment_format_map.md</t>
+          <t>https://tea.texas.gov/data-reports/staar/staar-english-ii-blueprint-schematic.pdf</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>03_state_assessment_format_map.md</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Maps every state's HS-writing assessment format onto the spine. Also cited under Category 2.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>03_state_assessment_format_map.md, 04_item_formats_and_rubrics.md</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>Texas Education Agency (TEA), STAAR Argumentative/Informational Rubrics</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>G9-12 Writing Assessment: Item Formats &amp; Scoring Rubrics</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>STAAR trait structure (Org &amp; Dev 0-3, Conv 0-2); dual-rater scoring, 10-point maximum</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://tea.texas.gov/data-reports/staar/tx-staar-arg-opinion-rubric-g6-e2.pdf</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>04_item_formats_and_rubrics.md</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\04_item_formats_and_rubrics.md</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>04_item_formats_and_rubrics.md</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Item taxonomy + rubric deep-dive per system (STAAR/Regents/SBAC/ACT/AP/NAEP), each traced to an official blueprint URL.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>College Board, AP English Language and Composition FRQ Scoring Rubrics</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Grade-10 ANCHOR Reference Forms — Full Released Forms + Scoring Guides + Annotated Student Work</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>G10_anchor_forms.md</t>
+          <t>AP Lang 6-point analytic rubric (Thesis 0-1, Evidence &amp; Commentary 0-4, Sophistication 0-1); applies to Synthesis, Rhetorical Analysis, Argument essays</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\AnchorSets\G10_anchor_forms.md</t>
+          <t>https://apcentral.collegeboard.org/media/pdf/ap-english-language-and-composition-frqs-1-2-3-scoring-rubrics.pdf</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>G10_anchor_forms.md</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>35</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Real G10 anchor forms (STAAR/MCAS/Regents) with annotated student work.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>04_item_formats_and_rubrics.md, G11_anchor_AP_Lang.md</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>College Board, AP English Literature and Composition FRQ Scoring Rubrics</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Grade-11 ANCHOR Reference — ACT Writing (Optional Essay)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>G11_anchor_ACT.md</t>
+          <t>AP Lit 6-point analytic rubric (parallel structure to AP Lang); applies to Poetry, Prose, Literary Argument essays</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\AnchorSets\G11_anchor_ACT.md</t>
+          <t>https://apcentral.collegeboard.org/media/pdf/ap-english-literature-and-composition-frqs-1-2-3-scoring-rubrics.pdf</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>G11_anchor_ACT.md</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>G11 anchor set: ACT Writing (3-perspective).</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>04_item_formats_and_rubrics.md, TestDesign_Reference.md</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>ACT, Inc., Description of ACT Writing Test</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Grade 11-12 ANCHOR Reference — AP English Language and Composition Free-Response (FRQ) Writing Tasks</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>G11_anchor_AP_Lang.md</t>
+          <t>ACT Writing 40-minute prompt (three perspectives); 4 analytic domains (Ideas and Analysis, Development and Support, Organization, Language Use and Conventions), each scored 1-6 by two raters, reported 2-12</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\AnchorSets\G11_anchor_AP_Lang.md</t>
+          <t>https://www.act.org/content/act/en/products-and-services/the-act/test-preparation/description-of-writing-test.html</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>G11_anchor_AP_Lang.md</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>G11 anchor set: AP English Language (synthesis / rhetorical analysis / argument).</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>03_state_assessment_format_map.md, 04_item_formats_and_rubrics.md</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>Smarter Balanced Assessment Consortium, Performance Task Writing Rubrics</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Grade-11 ANCHOR Reference — Smarter Balanced (SBAC) ELA/Literacy</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>G11_anchor_SBAC.md</t>
+          <t>SBAC G11 full-write rubric (Org/Purpose 1-4, Evidence/Elaboration 1-4, Conventions 0-2); argument and explanatory modes (no narrative G11)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\AnchorSets\G11_anchor_SBAC.md</t>
+          <t>https://portal.smarterbalanced.org/library/en/performance-task-writing-rubric-argumentative.pdf</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>G11_anchor_SBAC.md</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>16.1</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>G11 anchor set: SBAC full-write performance task.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>03_state_assessment_format_map.md, 04_item_formats_and_rubrics.md</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>New York State Education Department (NYSED), Regents Examination in ELA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>G9-12 Writing Test-Design Reference (from real released tests)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>TestDesign_Reference.md</t>
+          <t>NY Regents G11 two-essay format (source-based Argument 6-point, Text-Analysis Exposition 4-point); no discrete grammar section</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\TestDesign_Reference.md</t>
+          <t>https://www.nysedregents.org/hsela/</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TestDesign_Reference.md</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Compiled test-design spec from all 5 released-form batches; the grounding-against-real-forms trail.</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>03_state_assessment_format_map.md, 04_item_formats_and_rubrics.md, G10_anchor_forms.md</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>Massachusetts Department of Elementary and Secondary Education, MCAS Grade 10 Test Design</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>G9-12 Writing Test-Bank Blueprint — Reference-Corpus Spec (v1)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TestBank_Blueprint.md</t>
+          <t>MCAS G10 text-based essay (8-point rubric)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\TestBank_Blueprint.md</t>
+          <t>https://www.doe.mass.edu/mcas/tdd/testdesign/g10-ela.docx</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TestBank_Blueprint.md</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>14</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>The 4-layer reference-corpus spec (anchors / model lessons / stimuli / item spec).</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>03_state_assessment_format_map.md, G10_anchor_forms.md</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2. Exam Ground Truth (tested demands)</t>
+          <t>Florida Department of Education, B.E.S.T. Writing Argumentation Rubric</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Three Real G10 Forms vs. Exemplar — Structural Grounding</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>THREE_real_forms_vs_exemplar.html</t>
+          <t>FL B.E.S.T. G7-10 argumentation rubric; gating rule (no citation caps Development at 2/4)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\AnchorSets\THREE_real_forms_vs_exemplar.html</t>
+          <t>https://www.fldoe.org/file/20102/7-10BESTWritingArgumentationRubric.pdf</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>THREE_real_forms_vs_exemplar.html</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>11</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Browsable: our exemplars grounded against three real released forms.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>04_item_formats_and_rubrics.md, TestDesign_Reference.md</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Category 2: Exam Ground Truth</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Judith Hochman &amp; Natalie Wexler, The Writing Revolution (TWR)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Unit 1 Syntactic Moves: Inventory, Paired Errors, and Test Crosswalk</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>syntactic-moves-crosswalk.md</t>
+          <t>Sentence-level moves (because/but/so, appositives, subordinate clauses); explicit teaching of syntactic choices; kernel-expansion pedagogy</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\syntactic-moves-crosswalk.md</t>
+          <t>*The Writing Revolution* (Hochman &amp; Wexler, 2017); thewritingrevolution.org; Natalie Wexler on X (@natwexler) and *The Knowledge Gap*.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>syntactic-moves-crosswalk.md</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>The sentence-level crosswalk (Elaborate/Compress/Arrange/Control + the shadow-error family). Grounds SPOV Truth 4.</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>syntactic-moves-crosswalk.md, icm/stages/01-move-crosswalks/output/moves-claim.md</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Category 3: Move Decomposition</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Gerald Graff &amp; Cathy Birkenstein, They Say / I Say (TSIS)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Claim &amp; Thesis Moves: Inventory, Discriminations, and Test Crosswalk</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>moves-claim.md</t>
+          <t>Meta-commentary templates ("They say X, I say Y"); framing, conceding, responding moves; counterargument moves</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\stages\01-move-crosswalks\output\moves-claim.md</t>
+          <t>*They Say / I Say* (Graff &amp; Birkenstein, 5th ed.); wwnorton.com.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>moves-claim.md</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>9</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Claim crosswalk (13 moves): tier, discrimination, signature error, ACC/CCSS code, tests paid.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>syntactic-moves-crosswalk.md, KC_Map_and_Unit_Arch_G9-12.md</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Category 3: Move Decomposition</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Debra Myhill</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Evidence &amp; Source-Use Moves: Inventory, Discriminations, and Test Crosswalk</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>moves-evidence.md</t>
+          <t>Grammar-as-choice paradigm (stylistic manipulation of sentence structure); Exeter research on contextualized grammar instruction</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\stages\01-move-crosswalks\output\moves-evidence.md</t>
+          <t>*Essential Primary Grammar* (Myhill); Exeter grammar-as-choice research; Google Scholar: Debra Myhill.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>moves-evidence.md</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Evidence crosswalk (12 moves).</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>syntactic-moves-crosswalk.md, KC_Map_and_Unit_Arch_G9-12.md</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Category 3: Move Decomposition</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Jeff Anderson</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Reasoning &amp; Commentary Moves: Inventory, Discriminations, and Test Crosswalk</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>moves-reasoning.md</t>
+          <t>Mentor-text analysis (noticing author's choices); sentence imitation and manipulation; "What do you notice?" inquiry approach</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\stages\01-move-crosswalks\output\moves-reasoning.md</t>
+          <t>*Mechanically Inclined*, *Everyday Editing* (Anderson); Jeff Anderson on X (@writeguyjeff).</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>moves-reasoning.md</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Reasoning crosswalk (9 moves).</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>syntactic-moves-crosswalk.md, icm/stages/01-move-crosswalks/output/moves-revision.md</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Category 3: Move Decomposition</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Siegfried Engelmann, Theory of Instruction (Direct Instruction)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Organization &amp; Discourse Moves: Inventory, Discriminations, and Test Crosswalk</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>moves-organization.md</t>
+          <t>Discrimination-before-production pedagogy; minimal-pair contrasts; explicit sequence design. **(Grade-C / design bet, unvalidated for writing)** The discrimination-before-production principle is grounded in Engelmann's work on concept acquisition, but its application to essay-level compositional moves in this course is a design bet, not validated by direct empirical evidence in writing pedagogy.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\stages\01-move-crosswalks\output\moves-organization.md</t>
+          <t>*Theory of Instruction* (Engelmann &amp; Carnine); National Institute for Direct Instruction (nifdi.org).</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>moves-organization.md</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>7</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Organization crosswalk (10 moves).</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>pipeline/lesson_contract.py, LESSON_ARCHETYPES.html</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Category 4: Lesson Contract</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Barak Rosenshine, Principles of Instruction</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Revision &amp; Calibration Moves: Inventory, Discriminations, and Test Crosswalk</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>moves-revision.md</t>
+          <t>Check for understanding (CFU) after each small step; guided practice before independent practice; systematic review</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\stages\01-move-crosswalks\output\moves-revision.md</t>
+          <t>"Principles of Instruction" (Rosenshine, 2012, *American Educator*).</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>moves-revision.md</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Revision crosswalk (8 moves).</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>pipeline/lesson_contract.py, LESSON_ARCHETYPES.html</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Category 4: Lesson Contract</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Paul Kirschner, Carl Hendrick &amp; Jim Heal, How Learning Happens</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Task &amp; Genre-Decode Moves: Inventory, Discriminations, and Test Crosswalk</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>moves-task-decode.md</t>
+          <t>Cognitive load theory (novices need worked examples, not open-ended discovery); split-attention effect; expertise reversal effect (d=-0.43)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\stages\01-move-crosswalks\output\moves-task-decode.md</t>
+          <t>*How Learning Happens* (Kirschner, Hendrick &amp; Heal, 2020); Kirschner on X (@P_A_Kirschner).</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>moves-task-decode.md</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Task-decode crosswalk (6 moves).</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>pipeline/lesson_contract.py, LESSON_ARCHETYPES.html</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Category 4: Lesson Contract</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3. Move-Level Decomposition &amp; Crosswalks</t>
+          <t>Steve Graham &amp; Karen Harris, Self-Regulated Strategy Development (SRSD)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>G9-12 Writing KC Map + Unit Architectures (GAP-SCOPED, RECONCILED)</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KC_Map_and_Unit_Arch_G9-12.md</t>
+          <t>SRSD lesson shell (Develop Background Knowledge, Discuss, Model, Memorize, Support, Independent Practice); mnemonic strategy instruction; explicit teaching of planning and revision strategies</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\KC_Map_and_Unit_Arch_G9-12.md</t>
+          <t>srsdonline.org; Graham &amp; Perin, "Writing Next" (2007); *Powerful Writing Strategies for All Students* (Harris, Graham, Mason &amp; Friedlander, 2008); Google Scholar: Steve Graham (100,000+ citations).</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>KC_Map_and_Unit_Arch_G9-12.md</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>KC coding (Strand.Grade.Number; type D/P/S/I) and the move-&gt;KC trace. Also grounds Categories 6 &amp; 7.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>pipeline/lesson_contract.py, LESSON_ARCHETYPES.html, Lesson_Bank_G9/lesson_g9_l01_arguable_claim_v3_1.py</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Category 4: Lesson Contract</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4. Lesson Contract (SRSD shell, as code)</t>
+          <t>Paul Kirschner, Carl Hendrick &amp; Jim Heal, How Learning Happens</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>---- vocab -----------------------------------------------------------------</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>lesson_contract.py</t>
+          <t>Expertise reversal effect (scaffolding helps novices, d=+0.43; hurts experts, d=-0.43); fading protocol (withdraw worked examples as competence grows)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\pipeline\lesson_contract.py</t>
+          <t>*How Learning Happens* (Kirschner, Hendrick &amp; Heal, 2020); Kirschner on X (@P_A_Kirschner).</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>lesson_contract.py</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>62.7</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>The ~26 machine-enforced gates (shell completeness, discrimination-before-production, ladder, model sequence, calibration, etc.). Grounds SPOV Truths 3/6 and Myths 3/5.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>SPINE_DELIBERATION_verdict.md, SPINE_DELIBERATION_positions.md, Revision_Loop_Architecture.md</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Category 5: Fading, Transfer, and Calibration</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4. Lesson Contract (SRSD shell, as code)</t>
+          <t>Barry Zimmerman</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Lesson Archetype Catalog</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LESSON_ARCHETYPES.html</t>
+          <t>Self-regulated learning (SRL) progression (observation, emulation, self-control, self-regulation); metacognitive monitoring; gradual independence</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\LESSON_ARCHETYPES.html</t>
+          <t>Google Scholar: Barry Zimmerman (60,000+ citations); *Handbook of Self-Regulation of Learning and Performance* (Routledge, 2011).</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LESSON_ARCHETYPES.html</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Browsable: the 8 reusable archetypes (MARK/STAND/PROVE/DEW/CHECK/SPOT/BUILD/WEAVE) + mnemonic-honesty status.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>SPINE_DELIBERATION_verdict.md, Revision_Loop_Architecture.md</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Category 5: Fading, Transfer, and Calibration</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4. Lesson Contract (SRSD shell, as code)</t>
+          <t>Dylan Wiliam &amp; John Hattie</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>G10 Model-Lesson Specs (6 reusable types) — Council-Adjudicated v1</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>G10_Model_Lesson_Specs.md</t>
+          <t>Formative assessment and self-assessment calibration; rubric internalization; feedback loops</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\G10_Model_Lesson_Specs.md</t>
+          <t>*Embedded Formative Assessment* (Wiliam); *Visible Learning* (Hattie, 2009); Wiliam on X (@dylanwiliam).</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>G10_Model_Lesson_Specs.md</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>33.1</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>The model-lesson specs and council rulings encoded into gates. Grounds SPOV Truth 6, Myths 2/3.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Revision_Loop_Architecture.md, SPINE_DELIBERATION_verdict.md</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Category 5: Fading, Transfer, and Calibration</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4. Lesson Contract (SRSD shell, as code)</t>
+          <t>Steve Graham &amp; Karen Harris, SRSD</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>coping-model think-aloud panel: a WRITTEN drafting process (attempt -&gt; test -&gt; revise), then the endpoints.</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>lesson_g9_l01_arguable_claim_v3_1.py</t>
+          <t>SRSD fading sequence (Develop → Discuss → Model → Memorize → Support → Independent); gradual release of responsibility; transfer tasks</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\Lesson_Bank_G9\lesson_g9_l01_arguable_claim_v3_1.py</t>
+          <t>srsdonline.org; Graham &amp; Perin, "Writing Next" (2007); *Powerful Writing Strategies for All Students* (Harris, Graham, Mason &amp; Friedlander, 2008); Google Scholar: Steve Graham (100,000+ citations).</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>lesson_g9_l01_arguable_claim_v3_1.py</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>21</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>A live lesson instance (the coping panel with before/after) showing the contract realized.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>pipeline/lesson_contract.py, SPINE_DELIBERATION_verdict.md</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Category 5: Fading, Transfer, and Calibration</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5. Scaffold Fading, Transfer &amp; Calibration</t>
+          <t>David Yeager</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Lesson-spine deliberation: verdict + design (Council of Writing Instruction + Fable-5)</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SPINE_DELIBERATION_verdict.md</t>
+          <t>Adolescent motivation and growth mindset; self-transcendent purpose; mastery vs. performance goals; developmental context for G9-12 learners</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\SPINE_DELIBERATION_verdict.md</t>
+          <t>*10 to 25* (Yeager, 2024); Yeager on X (@dyeager1); Google Scholar: David Yeager.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SPINE_DELIBERATION_verdict.md</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>The grain-differentiated arc + scaffold-free-gate ruling (approved, mid-application). Grounds SPOV Truth 5 &amp; Insight 5.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>SPINE_DELIBERATION_positions.md, Revision_Loop_Architecture.md</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Category 5: Fading, Transfer, and Calibration</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5. Scaffold Fading, Transfer &amp; Calibration</t>
+          <t>Pietro Boscolo &amp; Suzanne Hidi</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Deliberations to adjudicate — 6 Council seats + Fable-5, on 3 lesson-architecture questions</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SPINE_DELIBERATION_positions.md</t>
+          <t>Writing motivation and interest; task value and self-efficacy; engagement in composition tasks</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\SPINE_DELIBERATION_positions.md</t>
+          <t>Hidi &amp; Boscolo, "Motivation and writing" (in *Handbook of Writing Research*); Boscolo &amp; Hidi, *Writing and Motivation* (2007).</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SPINE_DELIBERATION_positions.md</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>12.2</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>The council/Fable-5 positions behind the spine verdict.</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>SPINE_DELIBERATION_positions.md, COURSE_FIX_PLAN_synthesis.md</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Category 5: Fading, Transfer, and Calibration</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5. Scaffold Fading, Transfer &amp; Calibration</t>
+          <t>George Hillocks, Research on Written Composition</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Revision-Loop Architecture — Decision (to finalize lesson structures)</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Revision_Loop_Architecture.md</t>
+          <t>Grammar-in-isolation has near-zero effect on writing quality (d=-0.29 in 1986 meta-analysis); contextualized grammar instruction within real composition is effective</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\Revision_Loop_Architecture.md</t>
+          <t>*Research on Written Composition* (Hillocks, 1986); "The Testing Trap" (2002).</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Revision_Loop_Architecture.md</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>The revise-on-provided-pairs design (QTI is stateless).</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>KC_Map_and_Unit_Arch_G9-12.md, External_App_Scope.md</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Category 6: Scope and Ownership</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5. Scaffold Fading, Transfer &amp; Calibration</t>
+          <t>Debra Myhill</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HS Writing Course Fix Plan — synthesis of the two assessments</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COURSE_FIX_PLAN_synthesis.md</t>
+          <t>Grammar-as-choice paradigm (stylistic manipulation, not error-correction drills); Exeter research showing gains when grammar is taught as rhetorical resource in composition</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\COURSE_FIX_PLAN_synthesis.md</t>
+          <t>*Essential Primary Grammar* (Myhill); Exeter grammar-as-choice research; Google Scholar: Debra Myhill.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>COURSE_FIX_PLAN_synthesis.md</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>The calibration-loop honesty flag + the feedback-resolution #1 lever + Tier-4 BrainLift integration. Grounds Myths 5/6, Insight 10.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>KC_Map_and_Unit_Arch_G9-12.md, syntactic-moves-crosswalk.md</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Category 6: Scope and Ownership</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6. Scope Boundaries &amp; Course Ownership</t>
+          <t>Common Core State Standards (CCSS), Language Standards L.9-10.1-2 and L.11-12.1-2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>External Writing App — Scope &amp; Effort (Option E)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>External_App_Scope.md</t>
+          <t>Conventions standards (capitalization, punctuation, spelling, grammar, usage) across G9-12 band; scope and progression for CCSS-aligned states</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\External_App_Scope.md</t>
+          <t>https://www.cde.ca.gov/be/st/ss/documents/finalelaccssstandards.pdf</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>External_App_Scope.md</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Option E: the funded roadmap item that would enable true plan-draft-revise (not this deliverable).</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, KC_Map_and_Unit_Arch_G9-12.md</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Category 6: Scope and Ownership</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6. Scope Boundaries &amp; Course Ownership</t>
+          <t>Texas TEKS, Conventions Standards</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alpha HS Writing Course 2026-27 — Design &amp; Build Package</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>TEKS conventions scope (punctuation, capitalization, spelling, grammar) for English I/II; state-specific progression</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\README.md</t>
+          <t>https://tea.texas.gov/about-tea/laws-and-rules/texas-administrative-code/19-tac-chapter-110</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>README.md</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>The design/build package index + accepted-gap note (revise-your-own-work on stock QTI). Also grounds SPOV Truth 7.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>01_ccss_adherence_map.md, KC_Map_and_Unit_Arch_G9-12.md</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Category 6: Scope and Ownership</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
+          <t>Deborah McCutchen, "A capacity theory of writing: Working memory in composition"</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>G9-12 Course Scope &amp; Sequence</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SCOPE_SEQUENCE.html</t>
+          <t>Writing capacity theory (transcription, text generation, executive processes compete for limited working memory); novices struggle with simultaneous demands; supports chunking and fading</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\SCOPE_SEQUENCE.html</t>
+          <t>McCutchen, "A capacity theory of writing: Working memory in composition" (*Educational Psychology Review*, 1996); Google Scholar: Deborah McCutchen.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SCOPE_SEQUENCE.html</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Browsable: units -&gt; KCs -&gt; assessing items (the teaching map).</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>icm/CONTEXT.md, Revision_Loop_Architecture.md</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Category 7: Progression and Architecture</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
+          <t>John Hayes &amp; Linda Flower</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>G9-12 Lesson Allocation Map</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LESSON_MAP.html</t>
+          <t>Cognitive process model of writing (planning, translating, reviewing); recursive processes; expert-novice differences (experts plan more, revise more globally)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\LESSON_MAP.html</t>
+          <t>Hayes &amp; Flower, "A Cognitive Process Theory of Writing" (1981); Hayes, "A new framework for understanding cognition and affect in writing" (1996).</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>LESSON_MAP.html</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Browsable: KCs -&gt; ordered typed lessons + build-readiness.</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>icm/CONTEXT.md, KC_Map_and_Unit_Arch_G9-12.md</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Category 7: Progression and Architecture</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
+          <t>Grant Wiggins &amp; Jay McTighe, Understanding by Design (UbD)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>G9-12 Sentence-Skill Progression Map (VERIFIED, with assessment evidence)</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sentence_Progression_G9-12.md</t>
+          <t>Backward design (start with end-of-course assessment, design transfer tasks first, then build prerequisite skills); transfer as the goal</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\Sentence_Progression_G9-12.md</t>
+          <t>*Understanding by Design* (Wiggins &amp; McTighe, 2005); ASCD.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Sentence_Progression_G9-12.md</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>The G9-12 sentence progression.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>SCOPE_SEQUENCE.html, KC_Map_and_Unit_Arch_G9-12.md</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Category 7: Progression and Architecture</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
+          <t>Texas Education Agency (TEA), STAAR Blueprint (G9 English I, G10 English II)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Finalized HS Writing Skill Roster + Scaffold (G9-12) — GAP-SCOPED</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sentence_Skill_Roster_FINAL.md</t>
+          <t>Grade-to-exam map (G9 → STAAR English I, G10 → STAAR English II); ECR+SCR format anchors course endpoints</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\Sentence_Skill_Roster_FINAL.md</t>
+          <t>https://tea.texas.gov/data-reports/staar/staar-english-ii-blueprint-schematic.pdf</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sentence_Skill_Roster_FINAL.md</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>The finalized sentence-skill roster.</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>03_state_assessment_format_map.md, SCOPE_SEQUENCE.html</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Category 7: Progression and Architecture</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
+          <t>College Board, AP English Language Exam Structure</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Genre Spec: ARGUMENTATIVE (G9-G12)</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>genre-argumentative.md</t>
+          <t>G11 → AP Lang (Synthesis, Rhetorical Analysis, Argument FRQs); 6-point analytic rubric anchors G11 endpoint</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\stages\02-genre-specs\output\genre-argumentative.md</t>
+          <t>https://apcentral.collegeboard.org/media/pdf/ap-english-language-and-composition-frqs-1-2-3-scoring-rubrics.pdf</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>genre-argumentative.md</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>The argumentative genre spec (one of the 4). Grounds SPOV Truth 8.</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>03_state_assessment_format_map.md, 04_item_formats_and_rubrics.md</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Category 7: Progression and Architecture</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
+          <t>Peter Elbow &amp; Kelly Gallagher</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CONTEXT.md (Layer 1) - task routing</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CONTEXT.md</t>
+          <t>Process writing and authentic writing tasks; low-stakes writing; writing without teachers; writer's workshop; student choice and engagement</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\icm\CONTEXT.md</t>
+          <t>*Writing Without Teachers* (Elbow); *Write Like This* (Gallagher); Gallagher on X (@KellyGToGo).</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>CONTEXT.md</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>The ICM planned map / task routing (Layer 1).</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>LESSON_DESIGN_PLAN.md, icm/CONTEXT.md</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Category 7: Progression and Architecture</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
+          <t>Claim</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>G9-12 Writing Course - Build Dashboard</t>
+          <t>Authority</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DASHBOARD.html</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\DASHBOARD.html</t>
+          <t>Recovery type</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>DASHBOARD.html</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>12</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Browsable: the live control panel (coverage + QC status). Grounds Myths 4/7.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>7. Grade-Band Progression &amp; Architecture</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Lesson Design Plan: Scaffolding Audit + Authoring Principles</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>LESSON_DESIGN_PLAN.md</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\LESSON_DESIGN_PLAN.md</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>LESSON_DESIGN_PLAN.md</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Scaffolding audit + authoring principles + council rulings. Grounds SPOV Truths 7/8/9.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Cross-cutting (POVs / Insights)</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Alpha School HS Writing Courses</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>HS_Writing_Course_Blueprint.md</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>C:\Users\noelp\HS Writing\HS_Writing_Course_Blueprint.md</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>HS_Writing_Course_Blueprint.md</t>
-        </is>
-      </c>
-      <c r="F43" t="n">
-        <v>92.7</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>The master blueprint; source of the 4:2:1 plans:paragraphs:essays ratio (SPOV Myth 6). NOTE: lives in the HS Writing root, not the course folder.</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Cross-cutting (POVs / Insights)</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Retire Orphan Whole-Essay-Plan Lessons Implementation Plan</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>2026-07-17-retire-orphan-planning-lessons.md</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\docs\superpowers\plans\2026-07-17-retire-orphan-planning-lessons.md</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2026-07-17-retire-orphan-planning-lessons.md</t>
-        </is>
-      </c>
-      <c r="F44" t="n">
-        <v>17.2</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>The plan retiring orphan whole-essay-plan lessons (SPOV Myth 6 walk-back).</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Cross-cutting (POVs / Insights)</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>BrainLift Integration — what the HS Writing course can borrow, and what it's missing</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>BRAINLIFT_INTEGRATION.md</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>C:\Users\noelp\HS Writing\Alpha HS Writing Course 2026-27\BRAINLIFT_INTEGRATION.md</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>BRAINLIFT_INTEGRATION.md</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Companion audit of this design vs the Learning Scientists' BrainLift canon (borrow/gap findings, platform-split source).</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Category 7: Progression and Architecture</t>
         </is>
       </c>
     </row>

</xml_diff>